<commit_message>
Add internal APIs, NLU chat, and daily free-data tools so Streamlit Cloud can run the same desk.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/users.xlsx
+++ b/data/users.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,6 +471,55 @@
         <is>
           <t>ResetPending</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Hemant</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hemantchavan914@gmail.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>$2b$12$Z9eB2z5J9luvkSNs64IflOYJbdSgOAef0wRi4rqX1TYlg.Iye16g2</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:23:50Z</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:24:25Z</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-09-17T16:24:25Z</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>